<commit_message>
Fix role requirement in get_all_users
</commit_message>
<xml_diff>
--- a/Use Case Descriptions.xlsx
+++ b/Use Case Descriptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kelly\LOCAL_REPO\TPA-DESKTOP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B889B136-32EE-4C99-A9C4-D2613C4E7927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16176154-CC20-4562-BAA3-8C64DABEE66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="9" xr2:uid="{300492DA-25C7-4DE2-8F0D-49E1FFE71EA4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{300492DA-25C7-4DE2-8F0D-49E1FFE71EA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -865,40 +865,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -915,29 +882,122 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -945,110 +1005,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="22" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1398,153 +1398,153 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4"/>
+      <c r="D2" s="37"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="D3" s="37"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="37"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="39"/>
     </row>
     <row r="7" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="37"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="4"/>
+      <c r="D10" s="37"/>
     </row>
     <row r="11" spans="2:4" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="21"/>
+      <c r="D12" s="35"/>
     </row>
     <row r="13" spans="2:4" ht="0.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="13" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="19" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="6"/>
-      <c r="C16" s="19" t="s">
+      <c r="B16" s="27"/>
+      <c r="C16" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="7"/>
-      <c r="C17" s="20" t="s">
+      <c r="B17" s="28"/>
+      <c r="C17" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="17"/>
+      <c r="D18" s="6"/>
     </row>
     <row r="19" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32"/>
-      <c r="C19" s="18" t="s">
+      <c r="B19" s="34"/>
+      <c r="C19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="18"/>
+      <c r="D19" s="7"/>
     </row>
     <row r="20" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1590,105 +1590,105 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D4" s="43"/>
+      <c r="D4" s="29"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="10"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="21"/>
+      <c r="C14" s="5" t="s">
         <v>167</v>
       </c>
       <c r="D14" t="s">
@@ -1696,56 +1696,62 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="10"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="D15" s="38"/>
+      <c r="D15" s="10"/>
     </row>
     <row r="16" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="10"/>
-      <c r="C16" s="13" t="s">
+      <c r="B16" s="21"/>
+      <c r="C16" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="10" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="10"/>
-      <c r="C17" s="15" t="s">
+      <c r="B17" s="21"/>
+      <c r="C17" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="4" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="D18" s="34"/>
+      <c r="D18" s="23"/>
     </row>
     <row r="19" spans="2:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="28"/>
-      <c r="C19" s="22" t="s">
+      <c r="B19" s="11"/>
+      <c r="C19" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="23"/>
+      <c r="D19" s="18"/>
     </row>
     <row r="20" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="28"/>
-      <c r="C20" s="64" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="D20" s="65"/>
+      <c r="D20" s="20"/>
     </row>
     <row r="21" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="B13:B17"/>
@@ -1756,12 +1762,6 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1781,162 +1781,152 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="4"/>
+      <c r="D2" s="37"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="D3" s="37"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="37"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="39"/>
     </row>
     <row r="7" spans="2:4" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="37"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="4"/>
+      <c r="D10" s="37"/>
     </row>
     <row r="11" spans="2:4" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="37"/>
     </row>
     <row r="13" spans="2:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="7"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="28"/>
+      <c r="C15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="24"/>
+      <c r="D16" s="41"/>
     </row>
     <row r="17" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="27"/>
-      <c r="C17" s="24" t="s">
+      <c r="B17" s="42"/>
+      <c r="C17" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="24"/>
+      <c r="D17" s="41"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="27"/>
-      <c r="C18" s="25" t="s">
+      <c r="B18" s="42"/>
+      <c r="C18" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="25"/>
+      <c r="D18" s="40"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="27"/>
-      <c r="C19" s="13" t="s">
+      <c r="B19" s="42"/>
+      <c r="C19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="13"/>
+      <c r="D19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
@@ -1944,6 +1934,16 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="B16:B19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1963,166 +1963,156 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="25"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="28"/>
+      <c r="C16" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
     </row>
     <row r="18" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="35"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="43"/>
+      <c r="C18" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="D18" s="23"/>
+      <c r="D18" s="18"/>
     </row>
     <row r="19" spans="2:4" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32"/>
-      <c r="C19" s="22" t="s">
+      <c r="B19" s="34"/>
+      <c r="C19" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="23"/>
+      <c r="D19" s="18"/>
     </row>
     <row r="20" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
@@ -2130,6 +2120,16 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2149,164 +2149,154 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="25"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="28"/>
+      <c r="C16" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="10" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="35"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="43"/>
+      <c r="C18" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="23"/>
+      <c r="D18" s="18"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="32"/>
-      <c r="C19" s="22" t="s">
+      <c r="B19" s="34"/>
+      <c r="C19" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="23"/>
+      <c r="D19" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
@@ -2314,6 +2304,16 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2333,147 +2333,153 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="25"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="28"/>
+      <c r="C16" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="26"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="44"/>
+      <c r="C18" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="23"/>
+      <c r="D18" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C18:D18"/>
@@ -2484,12 +2490,6 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2509,143 +2509,147 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="40"/>
+      <c r="D4" s="46"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="42"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="48"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="38"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="10"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="26"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="44"/>
+      <c r="C18" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="23"/>
+      <c r="D18" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="C17:D17"/>
@@ -2657,10 +2661,6 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2680,154 +2680,159 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="43"/>
+      <c r="D4" s="29"/>
     </row>
     <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="6"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
+      <c r="B16" s="28"/>
       <c r="C16" t="s">
         <v>117</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="10" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="41" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="24"/>
+      <c r="D17" s="41"/>
     </row>
     <row r="18" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="26"/>
-      <c r="C18" s="24" t="s">
+      <c r="B18" s="44"/>
+      <c r="C18" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="24"/>
+      <c r="D18" s="41"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="26"/>
-      <c r="C19" s="13" t="s">
+      <c r="B19" s="44"/>
+      <c r="C19" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="13"/>
+      <c r="D19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C4:D4"/>
@@ -2839,11 +2844,6 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="B13:B16"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2863,164 +2863,168 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="25"/>
     </row>
     <row r="4" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="D4" s="40"/>
+      <c r="D4" s="46"/>
     </row>
     <row r="5" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="6"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="42"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="48"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="2:4" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="25"/>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="25"/>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="25"/>
     </row>
     <row r="11" spans="2:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="25"/>
     </row>
     <row r="12" spans="2:4" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="25"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="10"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="21"/>
+      <c r="C14" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="10"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="10" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="10"/>
-      <c r="C16" s="13" t="s">
+      <c r="B16" s="21"/>
+      <c r="C16" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D16" s="38"/>
+      <c r="D16" s="10"/>
     </row>
     <row r="17" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="13"/>
-      <c r="C17" s="13" t="s">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="4" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="13"/>
-      <c r="C18" s="13" t="s">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="4" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="D19" s="23"/>
+      <c r="D19" s="18"/>
     </row>
     <row r="20" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="30"/>
-      <c r="C20" s="22" t="s">
+      <c r="B20" s="50"/>
+      <c r="C20" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="D20" s="23"/>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C4:D5"/>
@@ -3032,10 +3036,6 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3052,7 +3052,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="58" t="s">
@@ -3061,7 +3061,7 @@
       <c r="D2" s="58"/>
     </row>
     <row r="3" spans="2:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="58" t="s">
@@ -3070,7 +3070,7 @@
       <c r="D3" s="58"/>
     </row>
     <row r="4" spans="2:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="64" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="58" t="s">
@@ -3079,17 +3079,17 @@
       <c r="D4" s="58"/>
     </row>
     <row r="5" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="59"/>
+      <c r="B5" s="64"/>
       <c r="C5" s="58"/>
       <c r="D5" s="58"/>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="59"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
     </row>
     <row r="7" spans="2:4" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="58" t="s">
@@ -3098,88 +3098,88 @@
       <c r="D7" s="58"/>
     </row>
     <row r="8" spans="2:4" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="59" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="50"/>
+      <c r="D8" s="60"/>
     </row>
     <row r="9" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="50"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="60"/>
     </row>
     <row r="10" spans="2:4" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="49" t="s">
+      <c r="C10" s="59" t="s">
         <v>147</v>
       </c>
-      <c r="D10" s="50"/>
+      <c r="D10" s="60"/>
     </row>
     <row r="11" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="49" t="s">
+      <c r="C11" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="D11" s="50"/>
+      <c r="D11" s="60"/>
     </row>
     <row r="12" spans="2:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="49" t="s">
+      <c r="C12" s="59" t="s">
         <v>149</v>
       </c>
-      <c r="D12" s="50"/>
+      <c r="D12" s="60"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="47" t="s">
+      <c r="D13" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="51"/>
-      <c r="C14" s="47" t="s">
+      <c r="B14" s="62"/>
+      <c r="C14" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D14" s="48" t="s">
+      <c r="D14" s="16" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="51"/>
-      <c r="C15" s="47" t="s">
+      <c r="B15" s="62"/>
+      <c r="C15" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="16" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="53"/>
-      <c r="C16" s="48" t="s">
+      <c r="B16" s="63"/>
+      <c r="C16" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="D16" s="48" t="s">
+      <c r="D16" s="16" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="51" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="54" t="s">
@@ -3188,14 +3188,14 @@
       <c r="D17" s="55"/>
     </row>
     <row r="18" spans="2:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="62"/>
+      <c r="B18" s="52"/>
       <c r="C18" s="54" t="s">
         <v>156</v>
       </c>
       <c r="D18" s="55"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="63"/>
+      <c r="B19" s="53"/>
       <c r="C19" s="56" t="s">
         <v>157</v>
       </c>
@@ -3203,6 +3203,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C18:D18"/>
@@ -3215,11 +3220,6 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="B13:B16"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>